<commit_message>
Moving ENMAK conditions to separate file
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_Base_VS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295E83BC-6C17-4947-9432-9178FD4E6147}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6328A232-9BF1-47D6-A4D2-2A6223C6EB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5220" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="re_targets" sheetId="5" r:id="rId1"/>
@@ -130,7 +130,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1686" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1666" uniqueCount="118">
   <si>
     <t>~TFM_INS-AT</t>
   </si>
@@ -488,57 +488,6 @@
   <si>
     <t>share_of_generation_pct</t>
   </si>
-  <si>
-    <t>Additions by Kristopher</t>
-  </si>
-  <si>
-    <t>PP_RENEW</t>
-  </si>
-  <si>
-    <t>Pset_Set</t>
-  </si>
-  <si>
-    <t>Pset_PN</t>
-  </si>
-  <si>
-    <t>Pset_CI</t>
-  </si>
-  <si>
-    <t>Pset_CO</t>
-  </si>
-  <si>
-    <t>Cset_CN</t>
-  </si>
-  <si>
-    <t>LimType</t>
-  </si>
-  <si>
-    <t>UC_FLO</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS</t>
-  </si>
-  <si>
-    <t>UC_RHSRTS~0</t>
-  </si>
-  <si>
-    <t>UC_Desc</t>
-  </si>
-  <si>
-    <t>ELC</t>
-  </si>
-  <si>
-    <t>LO</t>
-  </si>
-  <si>
-    <t>Minimum renewable power plants penetration</t>
-  </si>
-  <si>
-    <t>UC_min_renew_20235</t>
-  </si>
-  <si>
-    <t>~UC_T: UC_COMPRD</t>
-  </si>
 </sst>
 </file>
 
@@ -547,7 +496,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -615,20 +564,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <charset val="186"/>
-    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -689,7 +624,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -706,10 +641,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Heading 3" xfId="2" builtinId="18"/>
@@ -2116,28 +2047,22 @@
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="L17" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="18" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="L18" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="U18" s="14" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="20" spans="2:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>26</v>
       </c>
-      <c r="AC20" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="21" spans="2:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>27</v>
       </c>
@@ -2156,47 +2081,8 @@
       <c r="G21" t="s">
         <v>3</v>
       </c>
-      <c r="U21" s="16" t="s">
-        <v>13</v>
-      </c>
-      <c r="V21" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="W21" s="16" t="s">
-        <v>121</v>
-      </c>
-      <c r="X21" s="16" t="s">
-        <v>122</v>
-      </c>
-      <c r="Y21" s="16" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z21" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="AA21" s="16" t="s">
-        <v>56</v>
-      </c>
-      <c r="AB21" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="AC21" s="16" t="s">
-        <v>126</v>
-      </c>
-      <c r="AD21" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE21" s="16" t="s">
-        <v>127</v>
-      </c>
-      <c r="AF21" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="AG21" s="16" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="22" spans="2:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>32</v>
       </c>
@@ -2213,38 +2099,8 @@
       <c r="I22">
         <v>94</v>
       </c>
-      <c r="U22" t="s">
-        <v>133</v>
-      </c>
-      <c r="V22" t="s">
-        <v>119</v>
-      </c>
-      <c r="Z22" t="s">
-        <v>130</v>
-      </c>
-      <c r="AA22">
-        <v>2035</v>
-      </c>
-      <c r="AB22" t="s">
-        <v>131</v>
-      </c>
-      <c r="AC22" s="17">
-        <v>1</v>
-      </c>
-      <c r="AD22" s="15">
-        <v>-0.65</v>
-      </c>
-      <c r="AE22">
-        <v>0</v>
-      </c>
-      <c r="AF22">
-        <v>15</v>
-      </c>
-      <c r="AG22" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="23" spans="2:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>32</v>
       </c>
@@ -2261,10 +2117,8 @@
       <c r="I23">
         <v>55</v>
       </c>
-      <c r="AE23" s="15"/>
-      <c r="AF23" s="15"/>
-    </row>
-    <row r="24" spans="2:33" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>32</v>
       </c>
@@ -2282,7 +2136,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>44</v>
       </c>
@@ -2296,7 +2150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>44</v>
       </c>
@@ -2310,7 +2164,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="27" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>49</v>
       </c>
@@ -2325,7 +2179,7 @@
         <v>co2captured</v>
       </c>
     </row>
-    <row r="28" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>65</v>
       </c>
@@ -2336,7 +2190,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="2:33" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>67</v>
       </c>

</xml_diff>

<commit_message>
Adding Fermi's small nuclear power plant
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_Base_VS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6328A232-9BF1-47D6-A4D2-2A6223C6EB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09036EF4-2F32-4328-A7E1-98B1B894457F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="re_targets" sheetId="5" r:id="rId1"/>
@@ -1579,7 +1579,7 @@
     <col min="24" max="24" width="7.7109375" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="9.85546875" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="12" bestFit="1" customWidth="1"/>
@@ -2029,14 +2029,13 @@
       </c>
       <c r="AB15">
         <f>AE15*2.5</f>
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="AC15">
         <v>3</v>
       </c>
       <c r="AE15" s="11">
-        <f>SUMIFS(historical_data_long!$D$3:$D$626,historical_data_long!$A$3:$A$626,Veda!$V15,historical_data_long!$C$3:$C$626,"GW",historical_data_long!$B$3:$B$626,2022)</f>
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="AF15" s="10" t="s">
         <v>86</v>

</xml_diff>

<commit_message>
Removing base-year nuclear plant capacity
</commit_message>
<xml_diff>
--- a/VerveStacks_EST/SuppXLS/Scen_Base_VS.xlsx
+++ b/VerveStacks_EST/SuppXLS/Scen_Base_VS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\PycharmProjects\ee-times\VerveStacks_EST\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09036EF4-2F32-4328-A7E1-98B1B894457F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0075BAC7-DE6D-4D3B-B3C5-5E44DB93A023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-10470" yWindow="10890" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2029,13 +2029,13 @@
       </c>
       <c r="AB15">
         <f>AE15*2.5</f>
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="AC15">
         <v>3</v>
       </c>
       <c r="AE15" s="11">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="AF15" s="10" t="s">
         <v>86</v>

</xml_diff>